<commit_message>
guard: autosave 2026-08-24 17:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-08-24 16:55</t>
+          <t>생성: 2026-08-24 17:06</t>
         </is>
       </c>
     </row>
@@ -6691,7 +6691,7 @@
         <v>1010</v>
       </c>
       <c r="O62" s="8" t="n">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="P62" s="8" t="n">
         <v>820</v>
@@ -6700,13 +6700,13 @@
         <v>1430</v>
       </c>
       <c r="R62" s="8" t="n">
-        <v>1064</v>
+        <v>1076</v>
       </c>
       <c r="S62" s="8" t="n">
-        <v>940</v>
+        <v>945</v>
       </c>
       <c r="T62" s="8" t="n">
-        <v>962</v>
+        <v>964</v>
       </c>
       <c r="U62" s="8" t="n">
         <v>945</v>
@@ -10354,10 +10354,10 @@
         <v>-2.7</v>
       </c>
       <c r="N101" s="8" t="n">
-        <v>945</v>
+        <v>940</v>
       </c>
       <c r="O101" s="8" t="n">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="P101" s="8" t="n">
         <v>825</v>
@@ -30187,8 +30187,8 @@
       <c r="M312" s="7" t="n">
         <v>-1.1</v>
       </c>
-      <c r="N312" s="7" t="n">
-        <v>6</v>
+      <c r="N312" s="8" t="n">
+        <v>900</v>
       </c>
       <c r="O312" s="8" t="n">
         <v>353</v>
@@ -30217,8 +30217,8 @@
       <c r="W312" s="8" t="n">
         <v>1090</v>
       </c>
-      <c r="X312" s="7" t="n">
-        <v>6</v>
+      <c r="X312" s="8" t="n">
+        <v>900</v>
       </c>
       <c r="Y312" s="8" t="n">
         <v>496</v>
@@ -49600,7 +49600,7 @@
         <v>893</v>
       </c>
       <c r="AN518" s="8" t="n">
-        <v>999</v>
+        <v>666</v>
       </c>
     </row>
     <row r="519">
@@ -62906,7 +62906,7 @@
         <v>162</v>
       </c>
       <c r="P660" s="8" t="n">
-        <v>1040</v>
+        <v>1010</v>
       </c>
       <c r="Q660" s="8" t="n">
         <v>1390</v>

</xml_diff>

<commit_message>
guard: autosave 2026-08-25 08:30
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-08-24 17:18</t>
+          <t>생성: 2026-08-25 08:25</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY664"/>
+  <dimension ref="A1:AY665"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4753,7 +4753,7 @@
         <v>875</v>
       </c>
       <c r="AD41" s="8" t="n">
-        <v>1637</v>
+        <v>1632</v>
       </c>
       <c r="AE41" s="8" t="n">
         <v>1139</v>
@@ -9566,7 +9566,7 @@
         </is>
       </c>
       <c r="B93" s="7" t="n">
-        <v>82.5</v>
+        <v>83.3</v>
       </c>
       <c r="C93" s="7" t="n">
         <v>2</v>
@@ -9581,25 +9581,25 @@
         <v>676</v>
       </c>
       <c r="G93" s="7" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="H93" s="7" t="n">
         <v>5.3</v>
       </c>
       <c r="I93" s="7" t="n">
-        <v>-12.3</v>
+        <v>-12.1</v>
       </c>
       <c r="J93" s="7" t="n">
-        <v>10</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K93" s="7" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="L93" s="7" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="M93" s="7" t="n">
-        <v>-2.8</v>
+        <v>-2.5</v>
       </c>
       <c r="N93" s="8" t="n">
         <v>955</v>
@@ -11521,7 +11521,7 @@
         <v>925</v>
       </c>
       <c r="AD113" s="8" t="n">
-        <v>1718</v>
+        <v>1712</v>
       </c>
       <c r="AE113" s="8" t="n">
         <v>1120</v>
@@ -11614,9 +11614,6 @@
       <c r="Z114" s="8" t="n">
         <v>925</v>
       </c>
-      <c r="AD114" s="8" t="n">
-        <v>1712</v>
-      </c>
       <c r="AE114" s="8" t="n">
         <v>1135</v>
       </c>
@@ -11897,7 +11894,7 @@
         <v>925</v>
       </c>
       <c r="AD117" s="8" t="n">
-        <v>1691</v>
+        <v>1681</v>
       </c>
       <c r="AE117" s="8" t="n">
         <v>1150</v>
@@ -16127,7 +16124,7 @@
         <v>885</v>
       </c>
       <c r="AD162" s="8" t="n">
-        <v>1853</v>
+        <v>1830</v>
       </c>
       <c r="AE162" s="8" t="n">
         <v>1126</v>
@@ -30509,7 +30506,7 @@
         <v>860</v>
       </c>
       <c r="AD315" s="8" t="n">
-        <v>1761</v>
+        <v>1746</v>
       </c>
       <c r="AE315" s="8" t="n">
         <v>935</v>
@@ -50271,10 +50268,10 @@
         <v>68</v>
       </c>
       <c r="C526" s="7" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="D526" s="7" t="n">
-        <v>-0.6</v>
+        <v>-0.9</v>
       </c>
       <c r="E526" s="7" t="n">
         <v>64</v>
@@ -52599,7 +52596,7 @@
         <v>1180</v>
       </c>
       <c r="AD550" s="8" t="n">
-        <v>2026</v>
+        <v>1988</v>
       </c>
       <c r="AE550" s="8" t="n">
         <v>1338</v>
@@ -60119,7 +60116,7 @@
         <v>970</v>
       </c>
       <c r="AD630" s="8" t="n">
-        <v>2189</v>
+        <v>2219</v>
       </c>
       <c r="AE630" s="8" t="n">
         <v>941</v>
@@ -63325,6 +63322,73 @@
       </c>
       <c r="AN664" s="8" t="n">
         <v>840</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C665" s="7" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D665" s="7" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="F665" s="8" t="n">
+        <v>826</v>
+      </c>
+      <c r="N665" s="8" t="n">
+        <v>1050</v>
+      </c>
+      <c r="O665" s="8" t="n">
+        <v>225</v>
+      </c>
+      <c r="P665" s="8" t="n">
+        <v>1060</v>
+      </c>
+      <c r="Q665" s="8" t="n">
+        <v>1450</v>
+      </c>
+      <c r="R665" s="8" t="n">
+        <v>1011</v>
+      </c>
+      <c r="S665" s="8" t="n">
+        <v>951</v>
+      </c>
+      <c r="T665" s="8" t="n">
+        <v>955</v>
+      </c>
+      <c r="U665" s="8" t="n">
+        <v>1025</v>
+      </c>
+      <c r="V665" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="W665" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="X665" s="8" t="n">
+        <v>990</v>
+      </c>
+      <c r="Y665" s="8" t="n">
+        <v>730</v>
+      </c>
+      <c r="Z665" s="8" t="n">
+        <v>1105</v>
+      </c>
+      <c r="AD665" s="8" t="n">
+        <v>2416</v>
+      </c>
+      <c r="AE665" s="8" t="n">
+        <v>1206</v>
+      </c>
+      <c r="AM665" s="8" t="n">
+        <v>1076</v>
+      </c>
+      <c r="AN665" s="8" t="n">
+        <v>835</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
guard: autosave 2026-08-26 08:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-08-25 13:34</t>
+          <t>생성: 2026-08-26 08:02</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY665"/>
+  <dimension ref="A1:AY666"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -63330,6 +63330,9 @@
           <t>2026-08-24</t>
         </is>
       </c>
+      <c r="B665" s="7" t="n">
+        <v>97.90000000000001</v>
+      </c>
       <c r="C665" s="7" t="n">
         <v>-1.5</v>
       </c>
@@ -63342,6 +63345,27 @@
       <c r="F665" s="8" t="n">
         <v>826</v>
       </c>
+      <c r="G665" s="7" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="H665" s="7" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="I665" s="7" t="n">
+        <v>-8.300000000000001</v>
+      </c>
+      <c r="J665" s="7" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="K665" s="7" t="n">
+        <v>56</v>
+      </c>
+      <c r="L665" s="7" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="M665" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="N665" s="8" t="n">
         <v>1050</v>
       </c>
@@ -63391,6 +63415,100 @@
         <v>1076</v>
       </c>
       <c r="AN665" s="8" t="n">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B666" s="7" t="n">
+        <v>93</v>
+      </c>
+      <c r="C666" s="7" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D666" s="7" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="E666" s="7" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="F666" s="8" t="n">
+        <v>814</v>
+      </c>
+      <c r="G666" s="7" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="H666" s="7" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="I666" s="7" t="n">
+        <v>-5.1</v>
+      </c>
+      <c r="J666" s="7" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="K666" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="L666" s="7" t="n">
+        <v>61</v>
+      </c>
+      <c r="M666" s="7" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N666" s="8" t="n">
+        <v>1050</v>
+      </c>
+      <c r="O666" s="8" t="n">
+        <v>236</v>
+      </c>
+      <c r="P666" s="8" t="n">
+        <v>1060</v>
+      </c>
+      <c r="Q666" s="8" t="n">
+        <v>1450</v>
+      </c>
+      <c r="R666" s="8" t="n">
+        <v>1027</v>
+      </c>
+      <c r="S666" s="8" t="n">
+        <v>953</v>
+      </c>
+      <c r="T666" s="8" t="n">
+        <v>953</v>
+      </c>
+      <c r="U666" s="8" t="n">
+        <v>1025</v>
+      </c>
+      <c r="V666" s="8" t="n">
+        <v>211</v>
+      </c>
+      <c r="W666" s="8" t="n">
+        <v>1210</v>
+      </c>
+      <c r="X666" s="8" t="n">
+        <v>990</v>
+      </c>
+      <c r="Y666" s="8" t="n">
+        <v>745</v>
+      </c>
+      <c r="Z666" s="8" t="n">
+        <v>1105</v>
+      </c>
+      <c r="AD666" s="8" t="n">
+        <v>2416</v>
+      </c>
+      <c r="AE666" s="8" t="n">
+        <v>1221</v>
+      </c>
+      <c r="AM666" s="8" t="n">
+        <v>1078</v>
+      </c>
+      <c r="AN666" s="8" t="n">
         <v>835</v>
       </c>
     </row>

</xml_diff>

<commit_message>
guard: autosave 2026-08-27 08:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-08-26 09:30</t>
+          <t>생성: 2026-08-27 08:01</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY666"/>
+  <dimension ref="A1:AY667"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -63510,6 +63510,100 @@
       </c>
       <c r="AN666" s="8" t="n">
         <v>835</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B667" s="7" t="n">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="C667" s="7" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D667" s="7" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="E667" s="7" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="F667" s="8" t="n">
+        <v>797</v>
+      </c>
+      <c r="G667" s="7" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="H667" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="I667" s="7" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="J667" s="7" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="K667" s="7" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="L667" s="7" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="M667" s="7" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="N667" s="8" t="n">
+        <v>1030</v>
+      </c>
+      <c r="O667" s="8" t="n">
+        <v>233</v>
+      </c>
+      <c r="P667" s="8" t="n">
+        <v>1060</v>
+      </c>
+      <c r="Q667" s="8" t="n">
+        <v>1450</v>
+      </c>
+      <c r="R667" s="8" t="n">
+        <v>991</v>
+      </c>
+      <c r="S667" s="8" t="n">
+        <v>923</v>
+      </c>
+      <c r="T667" s="8" t="n">
+        <v>914</v>
+      </c>
+      <c r="U667" s="8" t="n">
+        <v>1025</v>
+      </c>
+      <c r="V667" s="8" t="n">
+        <v>228</v>
+      </c>
+      <c r="W667" s="8" t="n">
+        <v>1210</v>
+      </c>
+      <c r="X667" s="8" t="n">
+        <v>990</v>
+      </c>
+      <c r="Y667" s="8" t="n">
+        <v>680</v>
+      </c>
+      <c r="Z667" s="8" t="n">
+        <v>1105</v>
+      </c>
+      <c r="AD667" s="8" t="n">
+        <v>2421</v>
+      </c>
+      <c r="AE667" s="8" t="n">
+        <v>1181</v>
+      </c>
+      <c r="AM667" s="8" t="n">
+        <v>1039</v>
+      </c>
+      <c r="AN667" s="8" t="n">
+        <v>808</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
guard: autosave 2026-08-28 08:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-08-27 09:30</t>
+          <t>생성: 2026-08-28 08:01</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY667"/>
+  <dimension ref="A1:AY668"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -63604,6 +63604,100 @@
       </c>
       <c r="AN667" s="8" t="n">
         <v>808</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B668" s="7" t="n">
+        <v>90.40000000000001</v>
+      </c>
+      <c r="C668" s="7" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D668" s="7" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="E668" s="7" t="n">
+        <v>89.7</v>
+      </c>
+      <c r="F668" s="8" t="n">
+        <v>811</v>
+      </c>
+      <c r="G668" s="7" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="H668" s="7" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="I668" s="7" t="n">
+        <v>-3</v>
+      </c>
+      <c r="J668" s="7" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="K668" s="7" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="L668" s="7" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="M668" s="7" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="N668" s="8" t="n">
+        <v>1030</v>
+      </c>
+      <c r="O668" s="8" t="n">
+        <v>220</v>
+      </c>
+      <c r="P668" s="8" t="n">
+        <v>1060</v>
+      </c>
+      <c r="Q668" s="8" t="n">
+        <v>1450</v>
+      </c>
+      <c r="R668" s="8" t="n">
+        <v>1006</v>
+      </c>
+      <c r="S668" s="8" t="n">
+        <v>931</v>
+      </c>
+      <c r="T668" s="8" t="n">
+        <v>918</v>
+      </c>
+      <c r="U668" s="8" t="n">
+        <v>1025</v>
+      </c>
+      <c r="V668" s="8" t="n">
+        <v>215</v>
+      </c>
+      <c r="W668" s="8" t="n">
+        <v>1210</v>
+      </c>
+      <c r="X668" s="8" t="n">
+        <v>990</v>
+      </c>
+      <c r="Y668" s="8" t="n">
+        <v>680</v>
+      </c>
+      <c r="Z668" s="8" t="n">
+        <v>1105</v>
+      </c>
+      <c r="AD668" s="8" t="n">
+        <v>2428</v>
+      </c>
+      <c r="AE668" s="8" t="n">
+        <v>1191</v>
+      </c>
+      <c r="AM668" s="8" t="n">
+        <v>1046</v>
+      </c>
+      <c r="AN668" s="8" t="n">
+        <v>812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
guard: autosave 2026-08-28 09:40
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-08-28 08:01</t>
+          <t>생성: 2026-08-28 09:30</t>
         </is>
       </c>
     </row>
@@ -85766,16 +85766,16 @@
         <v>1000</v>
       </c>
       <c r="AR139" s="8" t="n">
+        <v>1330</v>
+      </c>
+      <c r="AS139" s="8" t="n">
         <v>1375</v>
       </c>
-      <c r="AS139" s="8" t="n">
-        <v>1400</v>
-      </c>
       <c r="AT139" s="8" t="n">
-        <v>2640</v>
+        <v>2605</v>
       </c>
       <c r="AU139" s="8" t="n">
-        <v>2595</v>
+        <v>2600</v>
       </c>
       <c r="AV139" s="8" t="n">
         <v>1215</v>

</xml_diff>

<commit_message>
guard: autosave 2026-08-31 08:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-08-30 09:30</t>
+          <t>생성: 2026-08-31 08:01</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY668"/>
+  <dimension ref="A1:AY669"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -63622,7 +63622,7 @@
         <v>-3.3</v>
       </c>
       <c r="E668" s="7" t="n">
-        <v>89.7</v>
+        <v>83.5</v>
       </c>
       <c r="F668" s="8" t="n">
         <v>811</v>
@@ -63698,6 +63698,100 @@
       </c>
       <c r="AN668" s="8" t="n">
         <v>812</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B669" s="7" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="C669" s="7" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D669" s="7" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="E669" s="7" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="F669" s="8" t="n">
+        <v>827</v>
+      </c>
+      <c r="G669" s="7" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="H669" s="7" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="I669" s="7" t="n">
+        <v>-4.1</v>
+      </c>
+      <c r="J669" s="7" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="K669" s="7" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="L669" s="7" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="M669" s="7" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="N669" s="8" t="n">
+        <v>1030</v>
+      </c>
+      <c r="O669" s="8" t="n">
+        <v>203</v>
+      </c>
+      <c r="P669" s="8" t="n">
+        <v>1060</v>
+      </c>
+      <c r="Q669" s="8" t="n">
+        <v>1450</v>
+      </c>
+      <c r="R669" s="8" t="n">
+        <v>1016</v>
+      </c>
+      <c r="S669" s="8" t="n">
+        <v>955</v>
+      </c>
+      <c r="T669" s="8" t="n">
+        <v>939</v>
+      </c>
+      <c r="U669" s="8" t="n">
+        <v>1025</v>
+      </c>
+      <c r="V669" s="8" t="n">
+        <v>198</v>
+      </c>
+      <c r="W669" s="8" t="n">
+        <v>1210</v>
+      </c>
+      <c r="X669" s="8" t="n">
+        <v>995</v>
+      </c>
+      <c r="Y669" s="8" t="n">
+        <v>690</v>
+      </c>
+      <c r="Z669" s="8" t="n">
+        <v>1105</v>
+      </c>
+      <c r="AD669" s="8" t="n">
+        <v>2440</v>
+      </c>
+      <c r="AE669" s="8" t="n">
+        <v>1208</v>
+      </c>
+      <c r="AM669" s="8" t="n">
+        <v>1065</v>
+      </c>
+      <c r="AN669" s="8" t="n">
+        <v>830</v>
       </c>
     </row>
   </sheetData>
@@ -63711,7 +63805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY139"/>
+  <dimension ref="A1:AY140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -85766,16 +85860,16 @@
         <v>1000</v>
       </c>
       <c r="AR139" s="8" t="n">
-        <v>1330</v>
+        <v>1375</v>
       </c>
       <c r="AS139" s="8" t="n">
-        <v>1375</v>
+        <v>1400</v>
       </c>
       <c r="AT139" s="8" t="n">
-        <v>2605</v>
+        <v>2640</v>
       </c>
       <c r="AU139" s="8" t="n">
-        <v>2600</v>
+        <v>2595</v>
       </c>
       <c r="AV139" s="8" t="n">
         <v>1215</v>
@@ -85788,6 +85882,163 @@
       </c>
       <c r="AY139" s="8" t="n">
         <v>1755</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-08 W4</t>
+        </is>
+      </c>
+      <c r="B140" s="7" t="n">
+        <v>92.3</v>
+      </c>
+      <c r="C140" s="7" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D140" s="7" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="E140" s="7" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="F140" s="8" t="n">
+        <v>815</v>
+      </c>
+      <c r="G140" s="7" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="H140" s="7" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="I140" s="7" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="J140" s="7" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="K140" s="7" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="L140" s="7" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="M140" s="7" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="N140" s="8" t="n">
+        <v>1038</v>
+      </c>
+      <c r="O140" s="8" t="n">
+        <v>223</v>
+      </c>
+      <c r="P140" s="8" t="n">
+        <v>1060</v>
+      </c>
+      <c r="Q140" s="8" t="n">
+        <v>1450</v>
+      </c>
+      <c r="R140" s="8" t="n">
+        <v>1010</v>
+      </c>
+      <c r="S140" s="8" t="n">
+        <v>942</v>
+      </c>
+      <c r="T140" s="8" t="n">
+        <v>935</v>
+      </c>
+      <c r="U140" s="8" t="n">
+        <v>1025</v>
+      </c>
+      <c r="V140" s="8" t="n">
+        <v>210</v>
+      </c>
+      <c r="W140" s="8" t="n">
+        <v>1208</v>
+      </c>
+      <c r="X140" s="8" t="n">
+        <v>991</v>
+      </c>
+      <c r="Y140" s="8" t="n">
+        <v>705</v>
+      </c>
+      <c r="Z140" s="8" t="n">
+        <v>1105</v>
+      </c>
+      <c r="AA140" s="8" t="n">
+        <v>1540</v>
+      </c>
+      <c r="AB140" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="AC140" s="8" t="n">
+        <v>2150</v>
+      </c>
+      <c r="AD140" s="8" t="n">
+        <v>2424</v>
+      </c>
+      <c r="AE140" s="8" t="n">
+        <v>1201</v>
+      </c>
+      <c r="AF140" s="8" t="n">
+        <v>1310</v>
+      </c>
+      <c r="AG140" s="8" t="n">
+        <v>1330</v>
+      </c>
+      <c r="AH140" s="8" t="n">
+        <v>1510</v>
+      </c>
+      <c r="AI140" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="AJ140" s="8" t="n">
+        <v>620</v>
+      </c>
+      <c r="AK140" s="8" t="n">
+        <v>385</v>
+      </c>
+      <c r="AL140" s="8" t="n">
+        <v>745</v>
+      </c>
+      <c r="AM140" s="8" t="n">
+        <v>1061</v>
+      </c>
+      <c r="AN140" s="8" t="n">
+        <v>824</v>
+      </c>
+      <c r="AO140" s="8" t="n">
+        <v>1045</v>
+      </c>
+      <c r="AP140" s="8" t="n">
+        <v>1095</v>
+      </c>
+      <c r="AQ140" s="8" t="n">
+        <v>1040</v>
+      </c>
+      <c r="AR140" s="8" t="n">
+        <v>1330</v>
+      </c>
+      <c r="AS140" s="8" t="n">
+        <v>1375</v>
+      </c>
+      <c r="AT140" s="8" t="n">
+        <v>2605</v>
+      </c>
+      <c r="AU140" s="8" t="n">
+        <v>2600</v>
+      </c>
+      <c r="AV140" s="8" t="n">
+        <v>1230</v>
+      </c>
+      <c r="AW140" s="8" t="n">
+        <v>1260</v>
+      </c>
+      <c r="AX140" s="8" t="n">
+        <v>1330</v>
+      </c>
+      <c r="AY140" s="8" t="n">
+        <v>1850</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
guard: autosave 2026-09-01 08:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-08-31 09:30</t>
+          <t>생성: 2026-09-01 08:01</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY669"/>
+  <dimension ref="A1:AY670"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -63792,6 +63792,100 @@
       </c>
       <c r="AN669" s="8" t="n">
         <v>830</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B670" s="7" t="n">
+        <v>95</v>
+      </c>
+      <c r="C670" s="7" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D670" s="7" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="E670" s="7" t="n">
+        <v>85.8</v>
+      </c>
+      <c r="F670" s="8" t="n">
+        <v>859</v>
+      </c>
+      <c r="G670" s="7" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="H670" s="7" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="I670" s="7" t="n">
+        <v>-2.4</v>
+      </c>
+      <c r="J670" s="7" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="K670" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="L670" s="7" t="n">
+        <v>59</v>
+      </c>
+      <c r="M670" s="7" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="N670" s="8" t="n">
+        <v>1080</v>
+      </c>
+      <c r="O670" s="8" t="n">
+        <v>221</v>
+      </c>
+      <c r="P670" s="8" t="n">
+        <v>1080</v>
+      </c>
+      <c r="Q670" s="8" t="n">
+        <v>1470</v>
+      </c>
+      <c r="R670" s="8" t="n">
+        <v>1066</v>
+      </c>
+      <c r="S670" s="8" t="n">
+        <v>990</v>
+      </c>
+      <c r="T670" s="8" t="n">
+        <v>984</v>
+      </c>
+      <c r="U670" s="8" t="n">
+        <v>1030</v>
+      </c>
+      <c r="V670" s="8" t="n">
+        <v>171</v>
+      </c>
+      <c r="W670" s="8" t="n">
+        <v>1270</v>
+      </c>
+      <c r="X670" s="8" t="n">
+        <v>1015</v>
+      </c>
+      <c r="Y670" s="8" t="n">
+        <v>735</v>
+      </c>
+      <c r="Z670" s="8" t="n">
+        <v>1115</v>
+      </c>
+      <c r="AD670" s="8" t="n">
+        <v>2440</v>
+      </c>
+      <c r="AE670" s="8" t="n">
+        <v>1268</v>
+      </c>
+      <c r="AM670" s="8" t="n">
+        <v>1111</v>
+      </c>
+      <c r="AN670" s="8" t="n">
+        <v>862</v>
       </c>
     </row>
   </sheetData>
@@ -86052,7 +86146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY35"/>
+  <dimension ref="A1:AY36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -91801,6 +91895,163 @@
       </c>
       <c r="AY35" s="8" t="n">
         <v>1674</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>88</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="F36" s="8" t="n">
+        <v>788</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="H36" s="7" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="J36" s="7" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="K36" s="7" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="L36" s="7" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="M36" s="7" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="N36" s="8" t="n">
+        <v>983</v>
+      </c>
+      <c r="O36" s="8" t="n">
+        <v>195</v>
+      </c>
+      <c r="P36" s="8" t="n">
+        <v>1038</v>
+      </c>
+      <c r="Q36" s="8" t="n">
+        <v>1368</v>
+      </c>
+      <c r="R36" s="8" t="n">
+        <v>967</v>
+      </c>
+      <c r="S36" s="8" t="n">
+        <v>932</v>
+      </c>
+      <c r="T36" s="8" t="n">
+        <v>938</v>
+      </c>
+      <c r="U36" s="8" t="n">
+        <v>1033</v>
+      </c>
+      <c r="V36" s="8" t="n">
+        <v>245</v>
+      </c>
+      <c r="W36" s="8" t="n">
+        <v>1182</v>
+      </c>
+      <c r="X36" s="8" t="n">
+        <v>968</v>
+      </c>
+      <c r="Y36" s="8" t="n">
+        <v>670</v>
+      </c>
+      <c r="Z36" s="8" t="n">
+        <v>1097</v>
+      </c>
+      <c r="AA36" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="AB36" s="8" t="n">
+        <v>1133</v>
+      </c>
+      <c r="AC36" s="8" t="n">
+        <v>2038</v>
+      </c>
+      <c r="AD36" s="8" t="n">
+        <v>2317</v>
+      </c>
+      <c r="AE36" s="8" t="n">
+        <v>1153</v>
+      </c>
+      <c r="AF36" s="8" t="n">
+        <v>1296</v>
+      </c>
+      <c r="AG36" s="8" t="n">
+        <v>1325</v>
+      </c>
+      <c r="AH36" s="8" t="n">
+        <v>1528</v>
+      </c>
+      <c r="AI36" s="8" t="n">
+        <v>323</v>
+      </c>
+      <c r="AJ36" s="8" t="n">
+        <v>605</v>
+      </c>
+      <c r="AK36" s="8" t="n">
+        <v>385</v>
+      </c>
+      <c r="AL36" s="8" t="n">
+        <v>751</v>
+      </c>
+      <c r="AM36" s="8" t="n">
+        <v>1068</v>
+      </c>
+      <c r="AN36" s="8" t="n">
+        <v>823</v>
+      </c>
+      <c r="AO36" s="8" t="n">
+        <v>1011</v>
+      </c>
+      <c r="AP36" s="8" t="n">
+        <v>1108</v>
+      </c>
+      <c r="AQ36" s="8" t="n">
+        <v>993</v>
+      </c>
+      <c r="AR36" s="8" t="n">
+        <v>1364</v>
+      </c>
+      <c r="AS36" s="8" t="n">
+        <v>1419</v>
+      </c>
+      <c r="AT36" s="8" t="n">
+        <v>2606</v>
+      </c>
+      <c r="AU36" s="8" t="n">
+        <v>2561</v>
+      </c>
+      <c r="AV36" s="8" t="n">
+        <v>1201</v>
+      </c>
+      <c r="AW36" s="8" t="n">
+        <v>1245</v>
+      </c>
+      <c r="AX36" s="8" t="n">
+        <v>1285</v>
+      </c>
+      <c r="AY36" s="8" t="n">
+        <v>1753</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
guard: autosave 2026-09-02 08:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-09-01 09:30</t>
+          <t>생성: 2026-09-02 08:01</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY670"/>
+  <dimension ref="A1:AY671"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -63886,6 +63886,100 @@
       </c>
       <c r="AN670" s="8" t="n">
         <v>862</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B671" s="7" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="C671" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D671" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E671" s="7" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="F671" s="8" t="n">
+        <v>849</v>
+      </c>
+      <c r="G671" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="H671" s="7" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="I671" s="7" t="n">
+        <v>-7.6</v>
+      </c>
+      <c r="J671" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="K671" s="7" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="L671" s="7" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="M671" s="7" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="N671" s="8" t="n">
+        <v>1115</v>
+      </c>
+      <c r="O671" s="8" t="n">
+        <v>267</v>
+      </c>
+      <c r="P671" s="8" t="n">
+        <v>1110</v>
+      </c>
+      <c r="Q671" s="8" t="n">
+        <v>1490</v>
+      </c>
+      <c r="R671" s="8" t="n">
+        <v>1056</v>
+      </c>
+      <c r="S671" s="8" t="n">
+        <v>1006</v>
+      </c>
+      <c r="T671" s="8" t="n">
+        <v>995</v>
+      </c>
+      <c r="U671" s="8" t="n">
+        <v>1040</v>
+      </c>
+      <c r="V671" s="8" t="n">
+        <v>192</v>
+      </c>
+      <c r="W671" s="8" t="n">
+        <v>1300</v>
+      </c>
+      <c r="X671" s="8" t="n">
+        <v>1025</v>
+      </c>
+      <c r="Y671" s="8" t="n">
+        <v>770</v>
+      </c>
+      <c r="Z671" s="8" t="n">
+        <v>1115</v>
+      </c>
+      <c r="AD671" s="8" t="n">
+        <v>2436</v>
+      </c>
+      <c r="AE671" s="8" t="n">
+        <v>1260</v>
+      </c>
+      <c r="AM671" s="8" t="n">
+        <v>1122</v>
+      </c>
+      <c r="AN671" s="8" t="n">
+        <v>870</v>
       </c>
     </row>
   </sheetData>
@@ -91907,10 +92001,10 @@
         <v>88</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>9.5</v>
+        <v>-1.5</v>
       </c>
       <c r="D36" s="7" t="n">
-        <v>7.8</v>
+        <v>-3.3</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>82.3</v>

</xml_diff>

<commit_message>
guard: autosave 2026-09-03 09:40
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-09-03 08:01</t>
+          <t>생성: 2026-09-03 09:30</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY671"/>
+  <dimension ref="A1:AY672"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -63980,6 +63980,100 @@
       </c>
       <c r="AN671" s="8" t="n">
         <v>870</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B672" s="8" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="C672" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D672" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E672" s="7" t="n">
+        <v>91</v>
+      </c>
+      <c r="F672" s="8" t="n">
+        <v>858</v>
+      </c>
+      <c r="G672" s="7" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="H672" s="7" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="I672" s="7" t="n">
+        <v>-9.300000000000001</v>
+      </c>
+      <c r="J672" s="7" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="K672" s="7" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="L672" s="7" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="M672" s="7" t="n">
+        <v>-7.9</v>
+      </c>
+      <c r="N672" s="8" t="n">
+        <v>1115</v>
+      </c>
+      <c r="O672" s="8" t="n">
+        <v>257</v>
+      </c>
+      <c r="P672" s="8" t="n">
+        <v>1120</v>
+      </c>
+      <c r="Q672" s="8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="R672" s="8" t="n">
+        <v>1085</v>
+      </c>
+      <c r="S672" s="8" t="n">
+        <v>1041</v>
+      </c>
+      <c r="T672" s="8" t="n">
+        <v>1013</v>
+      </c>
+      <c r="U672" s="8" t="n">
+        <v>1090</v>
+      </c>
+      <c r="V672" s="8" t="n">
+        <v>232</v>
+      </c>
+      <c r="W672" s="8" t="n">
+        <v>1325</v>
+      </c>
+      <c r="X672" s="8" t="n">
+        <v>1055</v>
+      </c>
+      <c r="Y672" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="Z672" s="8" t="n">
+        <v>1125</v>
+      </c>
+      <c r="AD672" s="8" t="n">
+        <v>2408</v>
+      </c>
+      <c r="AE672" s="8" t="n">
+        <v>1292</v>
+      </c>
+      <c r="AM672" s="8" t="n">
+        <v>1136</v>
+      </c>
+      <c r="AN672" s="8" t="n">
+        <v>881</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
guard: autosave 2026-09-04 08:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-09-03 09:30</t>
+          <t>생성: 2026-09-04 08:01</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY672"/>
+  <dimension ref="A1:AY673"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64074,6 +64074,100 @@
       </c>
       <c r="AN672" s="8" t="n">
         <v>881</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B673" s="8" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="C673" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D673" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E673" s="7" t="n">
+        <v>91.3</v>
+      </c>
+      <c r="F673" s="8" t="n">
+        <v>855</v>
+      </c>
+      <c r="G673" s="7" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="H673" s="7" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="I673" s="7" t="n">
+        <v>-9.699999999999999</v>
+      </c>
+      <c r="J673" s="7" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="K673" s="7" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="L673" s="7" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="M673" s="7" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="N673" s="8" t="n">
+        <v>1115</v>
+      </c>
+      <c r="O673" s="8" t="n">
+        <v>260</v>
+      </c>
+      <c r="P673" s="8" t="n">
+        <v>1120</v>
+      </c>
+      <c r="Q673" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="R673" s="8" t="n">
+        <v>1091</v>
+      </c>
+      <c r="S673" s="8" t="n">
+        <v>1071</v>
+      </c>
+      <c r="T673" s="8" t="n">
+        <v>1018</v>
+      </c>
+      <c r="U673" s="8" t="n">
+        <v>1080</v>
+      </c>
+      <c r="V673" s="8" t="n">
+        <v>225</v>
+      </c>
+      <c r="W673" s="8" t="n">
+        <v>1320</v>
+      </c>
+      <c r="X673" s="8" t="n">
+        <v>1055</v>
+      </c>
+      <c r="Y673" s="8" t="n">
+        <v>790</v>
+      </c>
+      <c r="Z673" s="8" t="n">
+        <v>1125</v>
+      </c>
+      <c r="AD673" s="8" t="n">
+        <v>2409</v>
+      </c>
+      <c r="AE673" s="8" t="n">
+        <v>1312</v>
+      </c>
+      <c r="AM673" s="8" t="n">
+        <v>1136</v>
+      </c>
+      <c r="AN673" s="8" t="n">
+        <v>880</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
guard: autosave 2026-09-07 08:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-09-06 09:30</t>
+          <t>생성: 2026-09-07 08:01</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY673"/>
+  <dimension ref="A1:AY674"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64170,6 +64170,100 @@
         <v>880</v>
       </c>
     </row>
+    <row r="674">
+      <c r="A674" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B674" s="8" t="n">
+        <v>101.9</v>
+      </c>
+      <c r="C674" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D674" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E674" s="7" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="F674" s="8" t="n">
+        <v>863</v>
+      </c>
+      <c r="G674" s="7" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="H674" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="I674" s="7" t="n">
+        <v>-9.1</v>
+      </c>
+      <c r="J674" s="7" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="K674" s="7" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="L674" s="7" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="M674" s="7" t="n">
+        <v>-7.8</v>
+      </c>
+      <c r="N674" s="8" t="n">
+        <v>1115</v>
+      </c>
+      <c r="O674" s="8" t="n">
+        <v>252</v>
+      </c>
+      <c r="P674" s="8" t="n">
+        <v>1120</v>
+      </c>
+      <c r="Q674" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="R674" s="8" t="n">
+        <v>1099</v>
+      </c>
+      <c r="S674" s="8" t="n">
+        <v>1064</v>
+      </c>
+      <c r="T674" s="8" t="n">
+        <v>1017</v>
+      </c>
+      <c r="U674" s="8" t="n">
+        <v>1070</v>
+      </c>
+      <c r="V674" s="8" t="n">
+        <v>207</v>
+      </c>
+      <c r="W674" s="8" t="n">
+        <v>1320</v>
+      </c>
+      <c r="X674" s="8" t="n">
+        <v>1055</v>
+      </c>
+      <c r="Y674" s="8" t="n">
+        <v>810</v>
+      </c>
+      <c r="Z674" s="8" t="n">
+        <v>1125</v>
+      </c>
+      <c r="AD674" s="8" t="n">
+        <v>2419</v>
+      </c>
+      <c r="AE674" s="8" t="n">
+        <v>1312</v>
+      </c>
+      <c r="AM674" s="8" t="n">
+        <v>1132</v>
+      </c>
+      <c r="AN674" s="8" t="n">
+        <v>876</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -64181,7 +64275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY140"/>
+  <dimension ref="A1:AY141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -86415,6 +86509,163 @@
       </c>
       <c r="AY140" s="8" t="n">
         <v>1850</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2026-09 W1</t>
+        </is>
+      </c>
+      <c r="B141" s="8" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="C141" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D141" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E141" s="7" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="F141" s="8" t="n">
+        <v>857</v>
+      </c>
+      <c r="G141" s="7" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="H141" s="7" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="I141" s="7" t="n">
+        <v>-7.6</v>
+      </c>
+      <c r="J141" s="7" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="K141" s="7" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="L141" s="7" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="M141" s="7" t="n">
+        <v>-6.3</v>
+      </c>
+      <c r="N141" s="8" t="n">
+        <v>1108</v>
+      </c>
+      <c r="O141" s="8" t="n">
+        <v>251</v>
+      </c>
+      <c r="P141" s="8" t="n">
+        <v>1110</v>
+      </c>
+      <c r="Q141" s="8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="R141" s="8" t="n">
+        <v>1079</v>
+      </c>
+      <c r="S141" s="8" t="n">
+        <v>1034</v>
+      </c>
+      <c r="T141" s="8" t="n">
+        <v>1005</v>
+      </c>
+      <c r="U141" s="8" t="n">
+        <v>1062</v>
+      </c>
+      <c r="V141" s="8" t="n">
+        <v>205</v>
+      </c>
+      <c r="W141" s="8" t="n">
+        <v>1307</v>
+      </c>
+      <c r="X141" s="8" t="n">
+        <v>1041</v>
+      </c>
+      <c r="Y141" s="8" t="n">
+        <v>781</v>
+      </c>
+      <c r="Z141" s="8" t="n">
+        <v>1121</v>
+      </c>
+      <c r="AA141" s="8" t="n">
+        <v>1535</v>
+      </c>
+      <c r="AB141" s="8" t="n">
+        <v>1240</v>
+      </c>
+      <c r="AC141" s="8" t="n">
+        <v>2180</v>
+      </c>
+      <c r="AD141" s="8" t="n">
+        <v>2422</v>
+      </c>
+      <c r="AE141" s="8" t="n">
+        <v>1289</v>
+      </c>
+      <c r="AF141" s="8" t="n">
+        <v>1360</v>
+      </c>
+      <c r="AG141" s="8" t="n">
+        <v>1410</v>
+      </c>
+      <c r="AH141" s="8" t="n">
+        <v>1550</v>
+      </c>
+      <c r="AI141" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="AJ141" s="8" t="n">
+        <v>620</v>
+      </c>
+      <c r="AK141" s="8" t="n">
+        <v>383</v>
+      </c>
+      <c r="AL141" s="8" t="n">
+        <v>765</v>
+      </c>
+      <c r="AM141" s="8" t="n">
+        <v>1127</v>
+      </c>
+      <c r="AN141" s="8" t="n">
+        <v>874</v>
+      </c>
+      <c r="AO141" s="8" t="n">
+        <v>1100</v>
+      </c>
+      <c r="AP141" s="8" t="n">
+        <v>1095</v>
+      </c>
+      <c r="AQ141" s="8" t="n">
+        <v>1050</v>
+      </c>
+      <c r="AR141" s="8" t="n">
+        <v>1350</v>
+      </c>
+      <c r="AS141" s="8" t="n">
+        <v>1495</v>
+      </c>
+      <c r="AT141" s="8" t="n">
+        <v>2565</v>
+      </c>
+      <c r="AU141" s="8" t="n">
+        <v>2570</v>
+      </c>
+      <c r="AV141" s="8" t="n">
+        <v>1255</v>
+      </c>
+      <c r="AW141" s="8" t="n">
+        <v>1300</v>
+      </c>
+      <c r="AX141" s="8" t="n">
+        <v>1370</v>
+      </c>
+      <c r="AY141" s="8" t="n">
+        <v>1915</v>
       </c>
     </row>
   </sheetData>

</xml_diff>